<commit_message>
Update tracker with 5 more documents (MD-089 to MD-093)
- MD-089 Cassar Ship Repair Ltd: Invoice 400215, Supply of Marble Sills, €106.20 incl VAT
- MD-090 May Grech: Delivery-Invoice 1000298, Supply of Marble for Penthouse, €436.60 incl VAT
- MD-091 Malta International Airport PLC: Delivery-Invoice 1000299 (Q299), Lime Stone Sills, €336.30 incl VAT
- MD-092 Stalagmite Connections: Invoice 400217, Marble Stair deposit €500.00 recorded
- MD-093 Blane: Quotation 317, Supply of Crema Marfil Sills, €551.65 incl VAT
- New clients C-040 to C-043 added to Client Directory with SUMIF formulas
- Blane Q317 added to Measurement Pipeline as L-040

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6MGCGosiZzZvgoKjqDuZ7
</commit_message>
<xml_diff>
--- a/MD_Marble_Factory_Tracker_Updated.xlsx
+++ b/MD_Marble_Factory_Tracker_Updated.xlsx
@@ -115,7 +115,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="910">
   <si>
     <t>MD MARBLE  —  FACTORY CONTROL DASHBOARD</t>
   </si>
@@ -2740,6 +2740,111 @@
   </si>
   <si>
     <t>L-039</t>
+  </si>
+  <si>
+    <t>MD-089</t>
+  </si>
+  <si>
+    <t>Cassar Ship Repair Ltd</t>
+  </si>
+  <si>
+    <t>Slip No 6 Cross Road, Marsa</t>
+  </si>
+  <si>
+    <t>Supply of Marble Sills</t>
+  </si>
+  <si>
+    <t>Marble Sills</t>
+  </si>
+  <si>
+    <t>VAT MT11461431 — Supply only — paid on delivery</t>
+  </si>
+  <si>
+    <t>MD-090</t>
+  </si>
+  <si>
+    <t>Marsaxlokk</t>
+  </si>
+  <si>
+    <t>Supply of Marble for Penthouse</t>
+  </si>
+  <si>
+    <t>Supply only — paid on delivery</t>
+  </si>
+  <si>
+    <t>MD-091</t>
+  </si>
+  <si>
+    <t>Malta International Airport PLC</t>
+  </si>
+  <si>
+    <t>Luqa LQA 4000</t>
+  </si>
+  <si>
+    <t>Supply &amp; Delivery of Lime Stone Sills (10m x 14cm + Delivery)</t>
+  </si>
+  <si>
+    <t>Lime Stone</t>
+  </si>
+  <si>
+    <t>MD-092</t>
+  </si>
+  <si>
+    <t>Stalagmite Connections</t>
+  </si>
+  <si>
+    <t>Mqabba</t>
+  </si>
+  <si>
+    <t>Supply of Marble Stair Fgura Etienne — Deposit</t>
+  </si>
+  <si>
+    <t>Marble Stair</t>
+  </si>
+  <si>
+    <t>VAT 18130814 — Deposit invoice — confirm received; full balance due on completion</t>
+  </si>
+  <si>
+    <t>MD-093</t>
+  </si>
+  <si>
+    <t>Blane</t>
+  </si>
+  <si>
+    <t>Santa Lucia</t>
+  </si>
+  <si>
+    <t>Supply of Crema Marfil Sills + Delivery, Santa Lucia</t>
+  </si>
+  <si>
+    <t>C-040</t>
+  </si>
+  <si>
+    <t>MT11461431</t>
+  </si>
+  <si>
+    <t>C-041</t>
+  </si>
+  <si>
+    <t>Corporate / Airport</t>
+  </si>
+  <si>
+    <t>C-042</t>
+  </si>
+  <si>
+    <t>18130814</t>
+  </si>
+  <si>
+    <t>C-043</t>
+  </si>
+  <si>
+    <t>L-040</t>
+  </si>
+  <si>
+    <t>Supply of Crema Marfil Sills + Delivery</t>
+  </si>
+  <si>
+    <t>Open quote — Santa Lucia</t>
   </si>
 </sst>
 </file>
@@ -9422,134 +9527,287 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="35"/>
-      <c r="B91" s="36"/>
-      <c r="C91" s="35"/>
-      <c r="D91" s="35"/>
-      <c r="E91" s="35"/>
-      <c r="F91" s="35"/>
-      <c r="G91" s="35"/>
-      <c r="H91" s="35"/>
-      <c r="I91" s="35"/>
-      <c r="J91" s="35"/>
-      <c r="K91" s="35"/>
-      <c r="L91" s="11"/>
-      <c r="M91" s="11"/>
-      <c r="N91" s="11"/>
-      <c r="O91" s="37"/>
-      <c r="P91" s="38" t="n">
-        <f aca="false">N91-O91</f>
+      <c r="A91" s="26" t="s">
+        <v>875</v>
+      </c>
+      <c r="B91" s="27">
+        <v>46070</v>
+      </c>
+      <c r="C91" s="28" t="s">
+        <v>876</v>
+      </c>
+      <c r="D91" s="28" t="s">
+        <v>877</v>
+      </c>
+      <c r="E91" s="29" t="s">
+        <v>878</v>
+      </c>
+      <c r="F91" s="28" t="s">
+        <v>879</v>
+      </c>
+      <c r="G91" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I91" s="26">
+        <v>400215</v>
+      </c>
+      <c r="J91" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K91" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="L91" s="30">
+        <v>90.0</v>
+      </c>
+      <c r="M91" s="30">
+        <v>16.2</v>
+      </c>
+      <c r="N91" s="30">
+        <v>106.2</v>
+      </c>
+      <c r="O91" s="31">
         <v>0</v>
       </c>
-      <c r="Q91" s="35"/>
-      <c r="R91" s="35"/>
-      <c r="S91" s="39"/>
-      <c r="T91" s="40"/>
-      <c r="U91" s="35"/>
+      <c r="P91" s="32">
+        <f>N91-O91</f>
+      </c>
+      <c r="Q91" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="R91" s="28" t="s">
+        <v>854</v>
+      </c>
+      <c r="U91" s="29" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="35"/>
-      <c r="B92" s="36"/>
-      <c r="C92" s="35"/>
-      <c r="D92" s="35"/>
-      <c r="E92" s="35"/>
-      <c r="F92" s="35"/>
-      <c r="G92" s="35"/>
-      <c r="H92" s="35"/>
-      <c r="I92" s="35"/>
-      <c r="J92" s="35"/>
-      <c r="K92" s="35"/>
-      <c r="L92" s="11"/>
-      <c r="M92" s="11"/>
-      <c r="N92" s="11"/>
-      <c r="O92" s="37"/>
-      <c r="P92" s="38" t="n">
-        <f aca="false">N92-O92</f>
+      <c r="A92" s="26" t="s">
+        <v>881</v>
+      </c>
+      <c r="B92" s="27">
+        <v>46070</v>
+      </c>
+      <c r="C92" s="28" t="s">
+        <v>433</v>
+      </c>
+      <c r="D92" s="28" t="s">
+        <v>882</v>
+      </c>
+      <c r="E92" s="29" t="s">
+        <v>883</v>
+      </c>
+      <c r="F92" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="G92" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="I92" s="26">
+        <v>1000298</v>
+      </c>
+      <c r="J92" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K92" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="L92" s="30">
+        <v>370.0</v>
+      </c>
+      <c r="M92" s="30">
+        <v>66.6</v>
+      </c>
+      <c r="N92" s="30">
+        <v>436.6</v>
+      </c>
+      <c r="O92" s="31">
         <v>0</v>
       </c>
-      <c r="Q92" s="35"/>
-      <c r="R92" s="35"/>
-      <c r="S92" s="39"/>
-      <c r="T92" s="40"/>
-      <c r="U92" s="35"/>
+      <c r="P92" s="32">
+        <f>N92-O92</f>
+      </c>
+      <c r="Q92" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="R92" s="28" t="s">
+        <v>854</v>
+      </c>
+      <c r="U92" s="29" t="s">
+        <v>884</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="35"/>
-      <c r="B93" s="36"/>
-      <c r="C93" s="35"/>
-      <c r="D93" s="35"/>
-      <c r="E93" s="35"/>
-      <c r="F93" s="35"/>
-      <c r="G93" s="35"/>
-      <c r="H93" s="35"/>
-      <c r="I93" s="35"/>
-      <c r="J93" s="35"/>
-      <c r="K93" s="35"/>
-      <c r="L93" s="11"/>
-      <c r="M93" s="11"/>
-      <c r="N93" s="11"/>
-      <c r="O93" s="37"/>
-      <c r="P93" s="38" t="n">
-        <f aca="false">N93-O93</f>
+      <c r="A93" s="26" t="s">
+        <v>885</v>
+      </c>
+      <c r="B93" s="27">
+        <v>46071</v>
+      </c>
+      <c r="C93" s="28" t="s">
+        <v>886</v>
+      </c>
+      <c r="D93" s="28" t="s">
+        <v>887</v>
+      </c>
+      <c r="E93" s="29" t="s">
+        <v>888</v>
+      </c>
+      <c r="F93" s="28" t="s">
+        <v>889</v>
+      </c>
+      <c r="G93" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H93" s="26">
+        <v>299</v>
+      </c>
+      <c r="I93" s="26">
+        <v>1000299</v>
+      </c>
+      <c r="J93" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K93" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="L93" s="30">
+        <v>285.0</v>
+      </c>
+      <c r="M93" s="30">
+        <v>51.3</v>
+      </c>
+      <c r="N93" s="30">
+        <v>336.3</v>
+      </c>
+      <c r="O93" s="31">
         <v>0</v>
       </c>
-      <c r="Q93" s="35"/>
-      <c r="R93" s="35"/>
-      <c r="S93" s="39"/>
-      <c r="T93" s="40"/>
-      <c r="U93" s="35"/>
+      <c r="P93" s="32">
+        <f>N93-O93</f>
+      </c>
+      <c r="Q93" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="R93" s="28" t="s">
+        <v>854</v>
+      </c>
+      <c r="U93" s="29" t="s">
+        <v>884</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="35"/>
-      <c r="B94" s="36"/>
-      <c r="C94" s="35"/>
-      <c r="D94" s="35"/>
-      <c r="E94" s="35"/>
-      <c r="F94" s="35"/>
-      <c r="G94" s="35"/>
-      <c r="H94" s="35"/>
-      <c r="I94" s="35"/>
-      <c r="J94" s="35"/>
-      <c r="K94" s="35"/>
-      <c r="L94" s="11"/>
-      <c r="M94" s="11"/>
-      <c r="N94" s="11"/>
-      <c r="O94" s="37"/>
-      <c r="P94" s="38" t="n">
-        <f aca="false">N94-O94</f>
+      <c r="A94" s="26" t="s">
+        <v>890</v>
+      </c>
+      <c r="B94" s="27">
+        <v>46074</v>
+      </c>
+      <c r="C94" s="28" t="s">
+        <v>891</v>
+      </c>
+      <c r="D94" s="28" t="s">
+        <v>892</v>
+      </c>
+      <c r="E94" s="29" t="s">
+        <v>893</v>
+      </c>
+      <c r="F94" s="28" t="s">
+        <v>894</v>
+      </c>
+      <c r="G94" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I94" s="26">
+        <v>400217</v>
+      </c>
+      <c r="J94" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K94" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="L94" s="30">
+        <v>423.73</v>
+      </c>
+      <c r="M94" s="30">
+        <v>76.27</v>
+      </c>
+      <c r="N94" s="30">
+        <v>500.0</v>
+      </c>
+      <c r="O94" s="31">
+        <v>500.0</v>
+      </c>
+      <c r="P94" s="32">
+        <f>N94-O94</f>
+      </c>
+      <c r="Q94" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R94" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="U94" s="29" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="26" t="s">
+        <v>896</v>
+      </c>
+      <c r="B95" s="27">
+        <v>46074</v>
+      </c>
+      <c r="C95" s="28" t="s">
+        <v>897</v>
+      </c>
+      <c r="D95" s="28" t="s">
+        <v>898</v>
+      </c>
+      <c r="E95" s="29" t="s">
+        <v>899</v>
+      </c>
+      <c r="F95" s="28" t="s">
+        <v>203</v>
+      </c>
+      <c r="G95" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H95" s="26">
+        <v>317</v>
+      </c>
+      <c r="J95" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K95" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="L95" s="30">
+        <v>467.5</v>
+      </c>
+      <c r="M95" s="30">
+        <v>84.15</v>
+      </c>
+      <c r="N95" s="30">
+        <v>551.65</v>
+      </c>
+      <c r="O95" s="31">
         <v>0</v>
       </c>
-      <c r="Q94" s="35"/>
-      <c r="R94" s="35"/>
-      <c r="S94" s="39"/>
-      <c r="T94" s="40"/>
-      <c r="U94" s="35"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="35"/>
-      <c r="B95" s="36"/>
-      <c r="C95" s="35"/>
-      <c r="D95" s="35"/>
-      <c r="E95" s="35"/>
-      <c r="F95" s="35"/>
-      <c r="G95" s="35"/>
-      <c r="H95" s="35"/>
-      <c r="I95" s="35"/>
-      <c r="J95" s="35"/>
-      <c r="K95" s="35"/>
-      <c r="L95" s="11"/>
-      <c r="M95" s="11"/>
-      <c r="N95" s="11"/>
-      <c r="O95" s="37"/>
-      <c r="P95" s="38" t="n">
-        <f aca="false">N95-O95</f>
-        <v>0</v>
-      </c>
-      <c r="Q95" s="35"/>
-      <c r="R95" s="35"/>
-      <c r="S95" s="39"/>
-      <c r="T95" s="40"/>
-      <c r="U95" s="35"/>
+      <c r="P95" s="32">
+        <f>N95-O95</f>
+      </c>
+      <c r="Q95" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R95" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="U95" s="29" t="s">
+        <v>863</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="35"/>
@@ -14140,24 +14398,168 @@
         <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B41,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B41,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H42" s="51" t="s">
+    <row r="42">
+      <c r="A42" s="17" t="s">
+        <v>900</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>876</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>901</v>
+      </c>
+      <c r="D42" s="20" t="s">
+        <v>877</v>
+      </c>
+      <c r="E42" s="43"/>
+      <c r="F42" s="19" t="s">
+        <v>483</v>
+      </c>
+      <c r="G42" s="44">
+        <v>46070</v>
+      </c>
+      <c r="H42" s="17">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B42)</f>
+      </c>
+      <c r="I42" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B42,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J42" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B42,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B42,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K42" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B42)</f>
+      </c>
+      <c r="L42" s="23">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B42,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B42,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="s">
+        <v>902</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>886</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>499</v>
+      </c>
+      <c r="D43" s="20" t="s">
+        <v>887</v>
+      </c>
+      <c r="E43" s="43"/>
+      <c r="F43" s="19" t="s">
+        <v>903</v>
+      </c>
+      <c r="G43" s="44">
+        <v>46071</v>
+      </c>
+      <c r="H43" s="17">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B43)</f>
+      </c>
+      <c r="I43" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B43,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J43" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B43,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B43,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K43" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B43)</f>
+      </c>
+      <c r="L43" s="23">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B43,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B43,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="s">
+        <v>904</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>891</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>905</v>
+      </c>
+      <c r="D44" s="20" t="s">
+        <v>892</v>
+      </c>
+      <c r="E44" s="43"/>
+      <c r="F44" s="19" t="s">
+        <v>483</v>
+      </c>
+      <c r="G44" s="44">
+        <v>46074</v>
+      </c>
+      <c r="H44" s="17">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B44)</f>
+      </c>
+      <c r="I44" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B44,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J44" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B44,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B44,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K44" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B44)</f>
+      </c>
+      <c r="L44" s="23">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B44,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B44,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="s">
+        <v>906</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>897</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>499</v>
+      </c>
+      <c r="D45" s="20" t="s">
+        <v>898</v>
+      </c>
+      <c r="E45" s="43"/>
+      <c r="F45" s="19" t="s">
+        <v>506</v>
+      </c>
+      <c r="G45" s="44">
+        <v>46074</v>
+      </c>
+      <c r="H45" s="17">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B45)</f>
+      </c>
+      <c r="I45" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J45" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K45" s="21">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B45)</f>
+      </c>
+      <c r="L45" s="23">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H46" s="51" t="s">
         <v>446</v>
       </c>
-      <c r="I42" s="52" t="n">
-        <f aca="false">SUM(I3:I41)</f>
+      <c r="I46" s="52" t="n">
+        <f aca="false">SUM(I3:I45)</f>
         <v>286888.31</v>
       </c>
-      <c r="J42" s="52" t="n">
-        <f aca="false">SUM(J3:J41)</f>
+      <c r="J46" s="52" t="n">
+        <f aca="false">SUM(J3:J45)</f>
         <v>139259.89</v>
       </c>
-      <c r="K42" s="52" t="n">
-        <f aca="false">SUM(K3:K41)</f>
+      <c r="K46" s="52" t="n">
+        <f aca="false">SUM(K3:K45)</f>
         <v>12372.58</v>
       </c>
-      <c r="L42" s="52" t="n">
-        <f aca="false">SUM(L3:L41)</f>
+      <c r="L46" s="52" t="n">
+        <f aca="false">SUM(L3:L45)</f>
         <v>126887.31</v>
       </c>
     </row>
@@ -15825,25 +16227,40 @@
         <v>863</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="35"/>
-      <c r="B42" s="36"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="40"/>
-      <c r="I42" s="35"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11" t="str">
-        <f aca="false">IF(J42="","",ROUND(J42*$R$2,2))</f>
-        <v/>
-      </c>
-      <c r="L42" s="35"/>
-      <c r="M42" s="39"/>
-      <c r="N42" s="40"/>
-      <c r="O42" s="35"/>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>907</v>
+      </c>
+      <c r="B42">
+        <v>46074</v>
+      </c>
+      <c r="C42" t="s">
+        <v>897</v>
+      </c>
+      <c r="E42" t="s">
+        <v>898</v>
+      </c>
+      <c r="F42" t="s">
+        <v>908</v>
+      </c>
+      <c r="G42" t="s">
+        <v>609</v>
+      </c>
+      <c r="I42">
+        <v>317</v>
+      </c>
+      <c r="J42">
+        <v>551.65</v>
+      </c>
+      <c r="K42">
+        <f>IF(J42="","",ROUND(J42*$R$2,2))</f>
+      </c>
+      <c r="L42" t="s">
+        <v>49</v>
+      </c>
+      <c r="O42" t="s">
+        <v>909</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="35"/>

</xml_diff>

<commit_message>
WIP: Add batch 3 docs and Price Book tab (in progress)
Partial update — agent still building Price Book tab and adding
MARSA Q318, JAA CO LTD, Gordon Vella Q323, BJORN Q324/Q325.
Final commit to follow on agent completion.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6MGCGosiZzZvgoKjqDuZ7
</commit_message>
<xml_diff>
--- a/MD_Marble_Factory_Tracker_Updated.xlsx
+++ b/MD_Marble_Factory_Tracker_Updated.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Attendance" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Workers" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Guide" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Price Book" sheetId="10" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Attendance!$A$2:$I$400</definedName>
@@ -115,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="910">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="1008">
   <si>
     <t>MD MARBLE  —  FACTORY CONTROL DASHBOARD</t>
   </si>
@@ -2845,6 +2846,300 @@
   </si>
   <si>
     <t>Open quote — Santa Lucia</t>
+  </si>
+  <si>
+    <t>MD-094</t>
+  </si>
+  <si>
+    <t>MD-095</t>
+  </si>
+  <si>
+    <t>MD-096</t>
+  </si>
+  <si>
+    <t>MD-097</t>
+  </si>
+  <si>
+    <t>MD-098</t>
+  </si>
+  <si>
+    <t>MARSA</t>
+  </si>
+  <si>
+    <t>Supply of Crema Galala Sills + Delivery</t>
+  </si>
+  <si>
+    <t>Quotation (Purchase Order)</t>
+  </si>
+  <si>
+    <t>Quote/Pending</t>
+  </si>
+  <si>
+    <t>Client name not on document — confirm client name</t>
+  </si>
+  <si>
+    <t>Arzella Xitwija, Triq Gizi, Swieqi</t>
+  </si>
+  <si>
+    <t>Supply of Marble Marsaskala</t>
+  </si>
+  <si>
+    <t>Gordon Vella</t>
+  </si>
+  <si>
+    <t>Supply of Light Travertine Sills (Sills, Stairs, Entrance)</t>
+  </si>
+  <si>
+    <t>Light Travertine</t>
+  </si>
+  <si>
+    <t>BJORN</t>
+  </si>
+  <si>
+    <t>Zabbar</t>
+  </si>
+  <si>
+    <t>Supply &amp; Install Bianco Marble &amp; Nero Assaluto</t>
+  </si>
+  <si>
+    <t>Bianco Marble / Nero Assaluto</t>
+  </si>
+  <si>
+    <t>Supply &amp; Install Quarzite &amp; Crema Marfil Marble (back light included with installation)</t>
+  </si>
+  <si>
+    <t>Quarzite / Crema Marfil</t>
+  </si>
+  <si>
+    <t>Open quote — back light included with installation; add to Measurement Pipeline</t>
+  </si>
+  <si>
+    <t>C-044</t>
+  </si>
+  <si>
+    <t>C-045</t>
+  </si>
+  <si>
+    <t>C-046</t>
+  </si>
+  <si>
+    <t>C-047</t>
+  </si>
+  <si>
+    <t>16456105</t>
+  </si>
+  <si>
+    <t>Corporate / TBC</t>
+  </si>
+  <si>
+    <t>L-041</t>
+  </si>
+  <si>
+    <t>L-042</t>
+  </si>
+  <si>
+    <t>L-043</t>
+  </si>
+  <si>
+    <t>L-044</t>
+  </si>
+  <si>
+    <t>Q318 — MARSA / Marsa</t>
+  </si>
+  <si>
+    <t>Q323 — Gordon Vella / Msida</t>
+  </si>
+  <si>
+    <t>Q324 — BJORN / Zabbar</t>
+  </si>
+  <si>
+    <t>Q325 — BJORN / Zabbar</t>
+  </si>
+  <si>
+    <t>Supply of Crema Galala Sills + Delivery — Open quote</t>
+  </si>
+  <si>
+    <t>Supply of Light Travertine Sills — Open quote</t>
+  </si>
+  <si>
+    <t>Supply &amp; Install Bianco Marble &amp; Nero Assaluto — Open quote</t>
+  </si>
+  <si>
+    <t>Supply &amp; Install Quarzite &amp; Crema Marfil — back light included</t>
+  </si>
+  <si>
+    <t>Quote/Pending — client name unconfirmed on document</t>
+  </si>
+  <si>
+    <t>Commercial</t>
+  </si>
+  <si>
+    <t>1000302</t>
+  </si>
+  <si>
+    <t>MD Marble — Client Price Book</t>
+  </si>
+  <si>
+    <t>Doc Ref</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Material / Item</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Unit Price (€)</t>
+  </si>
+  <si>
+    <t>Item Total (€)</t>
+  </si>
+  <si>
+    <t>ITIANA</t>
+  </si>
+  <si>
+    <t>VGP Property Investment Company Limited</t>
+  </si>
+  <si>
+    <t>Q324</t>
+  </si>
+  <si>
+    <t>Q325</t>
+  </si>
+  <si>
+    <t>Q317</t>
+  </si>
+  <si>
+    <t>Inv400215</t>
+  </si>
+  <si>
+    <t>Q323</t>
+  </si>
+  <si>
+    <t>Q310</t>
+  </si>
+  <si>
+    <t>1000296/Q306</t>
+  </si>
+  <si>
+    <t>1000299/Q299</t>
+  </si>
+  <si>
+    <t>Q318</t>
+  </si>
+  <si>
+    <t>1000298</t>
+  </si>
+  <si>
+    <t>Q309</t>
+  </si>
+  <si>
+    <t>Inv400217</t>
+  </si>
+  <si>
+    <t>1000290/Q303</t>
+  </si>
+  <si>
+    <t>Luqa</t>
+  </si>
+  <si>
+    <t>Nero Assaluto</t>
+  </si>
+  <si>
+    <t>Installation</t>
+  </si>
+  <si>
+    <t>Crema Marfil Sills</t>
+  </si>
+  <si>
+    <t>Light Travertine Sills</t>
+  </si>
+  <si>
+    <t>Light Travertine Stairs</t>
+  </si>
+  <si>
+    <t>Light Travertine Entrance</t>
+  </si>
+  <si>
+    <t>Supply of Stairs and Skirting (Beige)</t>
+  </si>
+  <si>
+    <t>Installation of Stairs and Skirting</t>
+  </si>
+  <si>
+    <t>Travertine (1st-2nd-3rd Floor)</t>
+  </si>
+  <si>
+    <t>Travertine (4th Floor)</t>
+  </si>
+  <si>
+    <t>Travertine (5th Floor)</t>
+  </si>
+  <si>
+    <t>Travertine (Ground Floor)</t>
+  </si>
+  <si>
+    <t>Travertine (Back Yard)</t>
+  </si>
+  <si>
+    <t>Lime Stone Sills 10m×14cm</t>
+  </si>
+  <si>
+    <t>Crema Galala Sills</t>
+  </si>
+  <si>
+    <t>Marble (Penthouse)</t>
+  </si>
+  <si>
+    <t>Bianco Carrara Roof Sills</t>
+  </si>
+  <si>
+    <t>Bianco Carrara Round Sills</t>
+  </si>
+  <si>
+    <t>Bianco Carrara Sills Level 1+2+3+4</t>
+  </si>
+  <si>
+    <t>Installation (all sills)</t>
+  </si>
+  <si>
+    <t>Marble Stair Fgura Etienne (deposit)</t>
+  </si>
+  <si>
+    <t>Bianco Carrera Sills</t>
+  </si>
+  <si>
+    <t>Extra Piece 2.40×25cm</t>
+  </si>
+  <si>
+    <t>Installation (incl. back light)</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>SQM</t>
+  </si>
+  <si>
+    <t>Lm</t>
+  </si>
+  <si>
+    <t>Back light included</t>
+  </si>
+  <si>
+    <t>Client name not confirmed on doc</t>
+  </si>
+  <si>
+    <t>Deposit invoice — full order TBC</t>
+  </si>
+  <si>
+    <t>Quarzite</t>
   </si>
 </sst>
 </file>
@@ -2862,7 +3157,7 @@
     <numFmt numFmtId="171" formatCode="hh:mm"/>
     <numFmt numFmtId="172" formatCode="\€#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2974,8 +3269,15 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3048,6 +3350,24 @@
         <bgColor rgb="FFD0D0D0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E4057"/>
+        <bgColor rgb="FF2E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFACD"/>
+        <bgColor rgb="FFFFFACD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -3098,7 +3418,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="79">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3386,6 +3706,27 @@
     <xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4109,6 +4450,1478 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FFFF8C00"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25" bestFit="true" customWidth="true"/>
+    <col min="2" max="2" width="15" customWidth="true"/>
+    <col min="3" max="3" width="12" customWidth="true"/>
+    <col min="4" max="4" width="20" customWidth="true"/>
+    <col min="5" max="5" width="30" customWidth="true"/>
+    <col min="6" max="6" width="8" customWidth="true"/>
+    <col min="7" max="7" width="10" customWidth="true"/>
+    <col min="8" max="8" width="14" customWidth="true"/>
+    <col min="9" max="9" width="14" customWidth="true"/>
+    <col min="10" max="10" width="15" customWidth="true"/>
+    <col min="11" max="11" width="30" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="true">
+      <c r="A1" s="72" t="s">
+        <v>953</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+    </row>
+    <row r="2" ht="18" customHeight="true">
+      <c r="A2" s="73" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="73" t="s">
+        <v>954</v>
+      </c>
+      <c r="C2" s="73" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="73" t="s">
+        <v>955</v>
+      </c>
+      <c r="E2" s="73" t="s">
+        <v>956</v>
+      </c>
+      <c r="F2" s="73" t="s">
+        <v>957</v>
+      </c>
+      <c r="G2" s="73" t="s">
+        <v>958</v>
+      </c>
+      <c r="H2" s="73" t="s">
+        <v>959</v>
+      </c>
+      <c r="I2" s="73" t="s">
+        <v>960</v>
+      </c>
+      <c r="J2" s="73" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="73" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="true">
+      <c r="A3" s="77" t="s">
+        <v>925</v>
+      </c>
+      <c r="B3" s="77" t="s">
+        <v>926</v>
+      </c>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+    </row>
+    <row r="4" ht="15" customHeight="true">
+      <c r="A4" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B4" s="74" t="s">
+        <v>963</v>
+      </c>
+      <c r="C4" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D4" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E4" s="74" t="s">
+        <v>977</v>
+      </c>
+      <c r="F4" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G4" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H4" s="76">
+        <v>1520.0</v>
+      </c>
+      <c r="I4" s="76">
+        <v>1520.0</v>
+      </c>
+      <c r="J4" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="74"/>
+    </row>
+    <row r="5" ht="15" customHeight="true">
+      <c r="A5" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B5" s="74" t="s">
+        <v>963</v>
+      </c>
+      <c r="C5" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D5" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E5" s="74" t="s">
+        <v>228</v>
+      </c>
+      <c r="F5" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G5" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H5" s="76">
+        <v>1680.0</v>
+      </c>
+      <c r="I5" s="76">
+        <v>1680.0</v>
+      </c>
+      <c r="J5" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="74"/>
+    </row>
+    <row r="6" ht="15" customHeight="true">
+      <c r="A6" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B6" s="74" t="s">
+        <v>963</v>
+      </c>
+      <c r="C6" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D6" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E6" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="F6" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G6" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H6" s="76">
+        <v>1100.0</v>
+      </c>
+      <c r="I6" s="76">
+        <v>1100.0</v>
+      </c>
+      <c r="J6" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K6" s="74"/>
+    </row>
+    <row r="7" ht="15" customHeight="true">
+      <c r="A7" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>964</v>
+      </c>
+      <c r="C7" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D7" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E7" s="74" t="s">
+        <v>203</v>
+      </c>
+      <c r="F7" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G7" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H7" s="76">
+        <v>960.0</v>
+      </c>
+      <c r="I7" s="76">
+        <v>960.0</v>
+      </c>
+      <c r="J7" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" s="74"/>
+    </row>
+    <row r="8" ht="15" customHeight="true">
+      <c r="A8" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B8" s="74" t="s">
+        <v>964</v>
+      </c>
+      <c r="C8" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D8" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E8" s="74" t="s">
+        <v>1007</v>
+      </c>
+      <c r="F8" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G8" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H8" s="76">
+        <v>4440.0</v>
+      </c>
+      <c r="I8" s="76">
+        <v>4440.0</v>
+      </c>
+      <c r="J8" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" s="74"/>
+    </row>
+    <row r="9" ht="15" customHeight="true">
+      <c r="A9" s="74" t="s">
+        <v>925</v>
+      </c>
+      <c r="B9" s="74" t="s">
+        <v>964</v>
+      </c>
+      <c r="C9" s="75">
+        <v>46079</v>
+      </c>
+      <c r="D9" s="74" t="s">
+        <v>926</v>
+      </c>
+      <c r="E9" s="74" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F9" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G9" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H9" s="76">
+        <v>1280.0</v>
+      </c>
+      <c r="I9" s="76">
+        <v>1280.0</v>
+      </c>
+      <c r="J9" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K9" s="74" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="true">
+      <c r="A10" s="77" t="s">
+        <v>897</v>
+      </c>
+      <c r="B10" s="77" t="s">
+        <v>898</v>
+      </c>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="77"/>
+      <c r="J10" s="77"/>
+      <c r="K10" s="77"/>
+    </row>
+    <row r="11" ht="15" customHeight="true">
+      <c r="A11" s="74" t="s">
+        <v>897</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>965</v>
+      </c>
+      <c r="C11" s="75">
+        <v>46074</v>
+      </c>
+      <c r="D11" s="74" t="s">
+        <v>898</v>
+      </c>
+      <c r="E11" s="74" t="s">
+        <v>979</v>
+      </c>
+      <c r="F11" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G11" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H11" s="76">
+        <v>427.5</v>
+      </c>
+      <c r="I11" s="76">
+        <v>427.5</v>
+      </c>
+      <c r="J11" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="74"/>
+    </row>
+    <row r="12" ht="15" customHeight="true">
+      <c r="A12" s="74" t="s">
+        <v>897</v>
+      </c>
+      <c r="B12" s="74" t="s">
+        <v>965</v>
+      </c>
+      <c r="C12" s="75">
+        <v>46074</v>
+      </c>
+      <c r="D12" s="74" t="s">
+        <v>898</v>
+      </c>
+      <c r="E12" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="F12" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G12" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H12" s="76">
+        <v>40.0</v>
+      </c>
+      <c r="I12" s="76">
+        <v>40.0</v>
+      </c>
+      <c r="J12" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="K12" s="74"/>
+    </row>
+    <row r="13" ht="15" customHeight="true">
+      <c r="A13" s="77" t="s">
+        <v>876</v>
+      </c>
+      <c r="B13" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="77"/>
+      <c r="K13" s="77"/>
+    </row>
+    <row r="14" ht="15" customHeight="true">
+      <c r="A14" s="74" t="s">
+        <v>876</v>
+      </c>
+      <c r="B14" s="74" t="s">
+        <v>966</v>
+      </c>
+      <c r="C14" s="75">
+        <v>46070</v>
+      </c>
+      <c r="D14" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="74" t="s">
+        <v>879</v>
+      </c>
+      <c r="F14" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G14" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H14" s="76">
+        <v>90.0</v>
+      </c>
+      <c r="I14" s="76">
+        <v>90.0</v>
+      </c>
+      <c r="J14" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14" s="74"/>
+    </row>
+    <row r="15" ht="15" customHeight="true">
+      <c r="A15" s="77" t="s">
+        <v>922</v>
+      </c>
+      <c r="B15" s="77" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="77"/>
+      <c r="F15" s="77"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="77"/>
+      <c r="I15" s="77"/>
+      <c r="J15" s="77"/>
+      <c r="K15" s="77"/>
+    </row>
+    <row r="16" ht="15" customHeight="true">
+      <c r="A16" s="74" t="s">
+        <v>922</v>
+      </c>
+      <c r="B16" s="74" t="s">
+        <v>967</v>
+      </c>
+      <c r="C16" s="75">
+        <v>46076</v>
+      </c>
+      <c r="D16" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E16" s="74" t="s">
+        <v>980</v>
+      </c>
+      <c r="F16" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G16" s="78">
+        <v>35.0</v>
+      </c>
+      <c r="H16" s="76">
+        <v>89.0</v>
+      </c>
+      <c r="I16" s="76">
+        <v>3115.0</v>
+      </c>
+      <c r="J16" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K16" s="74"/>
+    </row>
+    <row r="17" ht="15" customHeight="true">
+      <c r="A17" s="74" t="s">
+        <v>922</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>967</v>
+      </c>
+      <c r="C17" s="75">
+        <v>46076</v>
+      </c>
+      <c r="D17" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E17" s="74" t="s">
+        <v>981</v>
+      </c>
+      <c r="F17" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G17" s="78">
+        <v>165.0</v>
+      </c>
+      <c r="H17" s="76">
+        <v>89.0</v>
+      </c>
+      <c r="I17" s="76">
+        <v>14685.0</v>
+      </c>
+      <c r="J17" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" s="74"/>
+    </row>
+    <row r="18" ht="15" customHeight="true">
+      <c r="A18" s="74" t="s">
+        <v>922</v>
+      </c>
+      <c r="B18" s="74" t="s">
+        <v>967</v>
+      </c>
+      <c r="C18" s="75">
+        <v>46076</v>
+      </c>
+      <c r="D18" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E18" s="74" t="s">
+        <v>982</v>
+      </c>
+      <c r="F18" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G18" s="78">
+        <v>35.8</v>
+      </c>
+      <c r="H18" s="76">
+        <v>89.0</v>
+      </c>
+      <c r="I18" s="76">
+        <v>3186.2</v>
+      </c>
+      <c r="J18" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" s="74"/>
+    </row>
+    <row r="19" ht="15" customHeight="true">
+      <c r="A19" s="77" t="s">
+        <v>865</v>
+      </c>
+      <c r="B19" s="77" t="s">
+        <v>866</v>
+      </c>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
+      <c r="E19" s="77"/>
+      <c r="F19" s="77"/>
+      <c r="G19" s="77"/>
+      <c r="H19" s="77"/>
+      <c r="I19" s="77"/>
+      <c r="J19" s="77"/>
+      <c r="K19" s="77"/>
+    </row>
+    <row r="20" ht="15" customHeight="true">
+      <c r="A20" s="74" t="s">
+        <v>865</v>
+      </c>
+      <c r="B20" s="74" t="s">
+        <v>968</v>
+      </c>
+      <c r="C20" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D20" s="74" t="s">
+        <v>866</v>
+      </c>
+      <c r="E20" s="74" t="s">
+        <v>983</v>
+      </c>
+      <c r="F20" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G20" s="78">
+        <v>77.8</v>
+      </c>
+      <c r="H20" s="76">
+        <v>70.0</v>
+      </c>
+      <c r="I20" s="76">
+        <v>5446.0</v>
+      </c>
+      <c r="J20" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="74"/>
+    </row>
+    <row r="21" ht="15" customHeight="true">
+      <c r="A21" s="74" t="s">
+        <v>865</v>
+      </c>
+      <c r="B21" s="74" t="s">
+        <v>968</v>
+      </c>
+      <c r="C21" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D21" s="74" t="s">
+        <v>866</v>
+      </c>
+      <c r="E21" s="74" t="s">
+        <v>984</v>
+      </c>
+      <c r="F21" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G21" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H21" s="76">
+        <v>3890.0</v>
+      </c>
+      <c r="I21" s="76">
+        <v>3890.0</v>
+      </c>
+      <c r="J21" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K21" s="74"/>
+    </row>
+    <row r="22" ht="15" customHeight="true">
+      <c r="A22" s="77" t="s">
+        <v>961</v>
+      </c>
+      <c r="B22" s="77" t="s">
+        <v>424</v>
+      </c>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="77"/>
+    </row>
+    <row r="23" ht="15" customHeight="true">
+      <c r="A23" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B23" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C23" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D23" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E23" s="74" t="s">
+        <v>985</v>
+      </c>
+      <c r="F23" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G23" s="78">
+        <v>14.8</v>
+      </c>
+      <c r="H23" s="76">
+        <v>85.0</v>
+      </c>
+      <c r="I23" s="76">
+        <v>1258.0</v>
+      </c>
+      <c r="J23" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" s="74"/>
+    </row>
+    <row r="24" ht="15" customHeight="true">
+      <c r="A24" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B24" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C24" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D24" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E24" s="74" t="s">
+        <v>986</v>
+      </c>
+      <c r="F24" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G24" s="78">
+        <v>13.8</v>
+      </c>
+      <c r="H24" s="76">
+        <v>85.0</v>
+      </c>
+      <c r="I24" s="76">
+        <v>1173.0</v>
+      </c>
+      <c r="J24" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="74"/>
+    </row>
+    <row r="25" ht="15" customHeight="true">
+      <c r="A25" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B25" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C25" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D25" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E25" s="74" t="s">
+        <v>987</v>
+      </c>
+      <c r="F25" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G25" s="78">
+        <v>13.3</v>
+      </c>
+      <c r="H25" s="76">
+        <v>85.0</v>
+      </c>
+      <c r="I25" s="76">
+        <v>1130.5</v>
+      </c>
+      <c r="J25" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="74"/>
+    </row>
+    <row r="26" ht="15" customHeight="true">
+      <c r="A26" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B26" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C26" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D26" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E26" s="74" t="s">
+        <v>988</v>
+      </c>
+      <c r="F26" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G26" s="78">
+        <v>3.2</v>
+      </c>
+      <c r="H26" s="76">
+        <v>85.0</v>
+      </c>
+      <c r="I26" s="76">
+        <v>272.0</v>
+      </c>
+      <c r="J26" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="74"/>
+    </row>
+    <row r="27" ht="15" customHeight="true">
+      <c r="A27" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B27" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C27" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D27" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E27" s="74" t="s">
+        <v>989</v>
+      </c>
+      <c r="F27" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G27" s="78">
+        <v>8.3</v>
+      </c>
+      <c r="H27" s="76">
+        <v>85.0</v>
+      </c>
+      <c r="I27" s="76">
+        <v>705.5</v>
+      </c>
+      <c r="J27" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" s="74"/>
+    </row>
+    <row r="28" ht="15" customHeight="true">
+      <c r="A28" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B28" s="74" t="s">
+        <v>969</v>
+      </c>
+      <c r="C28" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D28" s="74" t="s">
+        <v>424</v>
+      </c>
+      <c r="E28" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="F28" s="74" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G28" s="78">
+        <v>217.0</v>
+      </c>
+      <c r="H28" s="76">
+        <v>15.0</v>
+      </c>
+      <c r="I28" s="76">
+        <v>3255.0</v>
+      </c>
+      <c r="J28" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K28" s="74"/>
+    </row>
+    <row r="29" ht="15" customHeight="true">
+      <c r="A29" s="77" t="s">
+        <v>200</v>
+      </c>
+      <c r="B29" s="77" t="s">
+        <v>201</v>
+      </c>
+      <c r="C29" s="77"/>
+      <c r="D29" s="77"/>
+      <c r="E29" s="77"/>
+      <c r="F29" s="77"/>
+      <c r="G29" s="77"/>
+      <c r="H29" s="77"/>
+      <c r="I29" s="77"/>
+      <c r="J29" s="77"/>
+      <c r="K29" s="77"/>
+    </row>
+    <row r="30" ht="15" customHeight="true">
+      <c r="A30" s="74" t="s">
+        <v>200</v>
+      </c>
+      <c r="B30" s="74" t="s">
+        <v>952</v>
+      </c>
+      <c r="C30" s="75">
+        <v>46078</v>
+      </c>
+      <c r="D30" s="74" t="s">
+        <v>201</v>
+      </c>
+      <c r="E30" s="74" t="s">
+        <v>921</v>
+      </c>
+      <c r="F30" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G30" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H30" s="76">
+        <v>13609.16</v>
+      </c>
+      <c r="I30" s="76">
+        <v>13609.16</v>
+      </c>
+      <c r="J30" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K30" s="74"/>
+    </row>
+    <row r="31" ht="15" customHeight="true">
+      <c r="A31" s="77" t="s">
+        <v>886</v>
+      </c>
+      <c r="B31" s="77" t="s">
+        <v>976</v>
+      </c>
+      <c r="C31" s="77"/>
+      <c r="D31" s="77"/>
+      <c r="E31" s="77"/>
+      <c r="F31" s="77"/>
+      <c r="G31" s="77"/>
+      <c r="H31" s="77"/>
+      <c r="I31" s="77"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="77"/>
+    </row>
+    <row r="32" ht="15" customHeight="true">
+      <c r="A32" s="74" t="s">
+        <v>886</v>
+      </c>
+      <c r="B32" s="74" t="s">
+        <v>970</v>
+      </c>
+      <c r="C32" s="75">
+        <v>46071</v>
+      </c>
+      <c r="D32" s="74" t="s">
+        <v>976</v>
+      </c>
+      <c r="E32" s="74" t="s">
+        <v>990</v>
+      </c>
+      <c r="F32" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G32" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H32" s="76">
+        <v>255.0</v>
+      </c>
+      <c r="I32" s="76">
+        <v>255.0</v>
+      </c>
+      <c r="J32" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K32" s="74"/>
+    </row>
+    <row r="33" ht="15" customHeight="true">
+      <c r="A33" s="74" t="s">
+        <v>886</v>
+      </c>
+      <c r="B33" s="74" t="s">
+        <v>970</v>
+      </c>
+      <c r="C33" s="75">
+        <v>46071</v>
+      </c>
+      <c r="D33" s="74" t="s">
+        <v>976</v>
+      </c>
+      <c r="E33" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="F33" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G33" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H33" s="76">
+        <v>30.0</v>
+      </c>
+      <c r="I33" s="76">
+        <v>30.0</v>
+      </c>
+      <c r="J33" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="K33" s="74"/>
+    </row>
+    <row r="34" ht="15" customHeight="true">
+      <c r="A34" s="77" t="s">
+        <v>915</v>
+      </c>
+      <c r="B34" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="77"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
+      <c r="I34" s="77"/>
+      <c r="J34" s="77"/>
+      <c r="K34" s="77"/>
+    </row>
+    <row r="35" ht="15" customHeight="true">
+      <c r="A35" s="74" t="s">
+        <v>915</v>
+      </c>
+      <c r="B35" s="74" t="s">
+        <v>971</v>
+      </c>
+      <c r="C35" s="75">
+        <v>46074</v>
+      </c>
+      <c r="D35" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="E35" s="74" t="s">
+        <v>991</v>
+      </c>
+      <c r="F35" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G35" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H35" s="76">
+        <v>337.5</v>
+      </c>
+      <c r="I35" s="76">
+        <v>337.5</v>
+      </c>
+      <c r="J35" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K35" s="74" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="true">
+      <c r="A36" s="74" t="s">
+        <v>915</v>
+      </c>
+      <c r="B36" s="74" t="s">
+        <v>971</v>
+      </c>
+      <c r="C36" s="75">
+        <v>46074</v>
+      </c>
+      <c r="D36" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="E36" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="F36" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G36" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H36" s="76">
+        <v>50.0</v>
+      </c>
+      <c r="I36" s="76">
+        <v>50.0</v>
+      </c>
+      <c r="J36" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="K36" s="74"/>
+    </row>
+    <row r="37" ht="15" customHeight="true">
+      <c r="A37" s="77" t="s">
+        <v>433</v>
+      </c>
+      <c r="B37" s="77" t="s">
+        <v>882</v>
+      </c>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
+      <c r="I37" s="77"/>
+      <c r="J37" s="77"/>
+      <c r="K37" s="77"/>
+    </row>
+    <row r="38" ht="15" customHeight="true">
+      <c r="A38" s="74" t="s">
+        <v>433</v>
+      </c>
+      <c r="B38" s="74" t="s">
+        <v>972</v>
+      </c>
+      <c r="C38" s="75">
+        <v>46070</v>
+      </c>
+      <c r="D38" s="74" t="s">
+        <v>882</v>
+      </c>
+      <c r="E38" s="74" t="s">
+        <v>992</v>
+      </c>
+      <c r="F38" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G38" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H38" s="76">
+        <v>370.0</v>
+      </c>
+      <c r="I38" s="76">
+        <v>370.0</v>
+      </c>
+      <c r="J38" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K38" s="74"/>
+    </row>
+    <row r="39" ht="15" customHeight="true">
+      <c r="A39" s="77" t="s">
+        <v>859</v>
+      </c>
+      <c r="B39" s="77" t="s">
+        <v>163</v>
+      </c>
+      <c r="C39" s="77"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
+      <c r="I39" s="77"/>
+      <c r="J39" s="77"/>
+      <c r="K39" s="77"/>
+    </row>
+    <row r="40" ht="15" customHeight="true">
+      <c r="A40" s="74" t="s">
+        <v>859</v>
+      </c>
+      <c r="B40" s="74" t="s">
+        <v>973</v>
+      </c>
+      <c r="C40" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D40" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E40" s="74" t="s">
+        <v>993</v>
+      </c>
+      <c r="F40" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G40" s="78">
+        <v>22.4</v>
+      </c>
+      <c r="H40" s="76">
+        <v>80.0</v>
+      </c>
+      <c r="I40" s="76">
+        <v>1792.0</v>
+      </c>
+      <c r="J40" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K40" s="74"/>
+    </row>
+    <row r="41" ht="15" customHeight="true">
+      <c r="A41" s="74" t="s">
+        <v>859</v>
+      </c>
+      <c r="B41" s="74" t="s">
+        <v>973</v>
+      </c>
+      <c r="C41" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D41" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E41" s="74" t="s">
+        <v>994</v>
+      </c>
+      <c r="F41" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G41" s="78">
+        <v>47.7</v>
+      </c>
+      <c r="H41" s="76">
+        <v>80.0</v>
+      </c>
+      <c r="I41" s="76">
+        <v>3816.0</v>
+      </c>
+      <c r="J41" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K41" s="74"/>
+    </row>
+    <row r="42" ht="15" customHeight="true">
+      <c r="A42" s="74" t="s">
+        <v>859</v>
+      </c>
+      <c r="B42" s="74" t="s">
+        <v>973</v>
+      </c>
+      <c r="C42" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D42" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E42" s="74" t="s">
+        <v>995</v>
+      </c>
+      <c r="F42" s="74" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G42" s="78">
+        <v>55.3</v>
+      </c>
+      <c r="H42" s="76">
+        <v>80.0</v>
+      </c>
+      <c r="I42" s="76">
+        <v>4424.0</v>
+      </c>
+      <c r="J42" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K42" s="74"/>
+    </row>
+    <row r="43" ht="15" customHeight="true">
+      <c r="A43" s="74" t="s">
+        <v>859</v>
+      </c>
+      <c r="B43" s="74" t="s">
+        <v>973</v>
+      </c>
+      <c r="C43" s="75">
+        <v>46067</v>
+      </c>
+      <c r="D43" s="74" t="s">
+        <v>163</v>
+      </c>
+      <c r="E43" s="74" t="s">
+        <v>996</v>
+      </c>
+      <c r="F43" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G43" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H43" s="76">
+        <v>5171.0</v>
+      </c>
+      <c r="I43" s="76">
+        <v>5171.0</v>
+      </c>
+      <c r="J43" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K43" s="74"/>
+    </row>
+    <row r="44" ht="15" customHeight="true">
+      <c r="A44" s="77" t="s">
+        <v>891</v>
+      </c>
+      <c r="B44" s="77" t="s">
+        <v>892</v>
+      </c>
+      <c r="C44" s="77"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
+      <c r="I44" s="77"/>
+      <c r="J44" s="77"/>
+      <c r="K44" s="77"/>
+    </row>
+    <row r="45" ht="15" customHeight="true">
+      <c r="A45" s="74" t="s">
+        <v>891</v>
+      </c>
+      <c r="B45" s="74" t="s">
+        <v>974</v>
+      </c>
+      <c r="C45" s="75">
+        <v>46074</v>
+      </c>
+      <c r="D45" s="74" t="s">
+        <v>892</v>
+      </c>
+      <c r="E45" s="74" t="s">
+        <v>997</v>
+      </c>
+      <c r="F45" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G45" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H45" s="76">
+        <v>423.73</v>
+      </c>
+      <c r="I45" s="76">
+        <v>423.73</v>
+      </c>
+      <c r="J45" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K45" s="74" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="true">
+      <c r="A46" s="77" t="s">
+        <v>962</v>
+      </c>
+      <c r="B46" s="77" t="s">
+        <v>429</v>
+      </c>
+      <c r="C46" s="77"/>
+      <c r="D46" s="77"/>
+      <c r="E46" s="77"/>
+      <c r="F46" s="77"/>
+      <c r="G46" s="77"/>
+      <c r="H46" s="77"/>
+      <c r="I46" s="77"/>
+      <c r="J46" s="77"/>
+      <c r="K46" s="77"/>
+    </row>
+    <row r="47" ht="15" customHeight="true">
+      <c r="A47" s="74" t="s">
+        <v>962</v>
+      </c>
+      <c r="B47" s="74" t="s">
+        <v>975</v>
+      </c>
+      <c r="C47" s="75">
+        <v>46065</v>
+      </c>
+      <c r="D47" s="74" t="s">
+        <v>429</v>
+      </c>
+      <c r="E47" s="74" t="s">
+        <v>998</v>
+      </c>
+      <c r="F47" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G47" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H47" s="76">
+        <v>349.5</v>
+      </c>
+      <c r="I47" s="76">
+        <v>349.5</v>
+      </c>
+      <c r="J47" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K47" s="74"/>
+    </row>
+    <row r="48" ht="15" customHeight="true">
+      <c r="A48" s="74" t="s">
+        <v>962</v>
+      </c>
+      <c r="B48" s="74" t="s">
+        <v>975</v>
+      </c>
+      <c r="C48" s="75">
+        <v>46065</v>
+      </c>
+      <c r="D48" s="74" t="s">
+        <v>429</v>
+      </c>
+      <c r="E48" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="F48" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G48" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H48" s="76">
+        <v>198.0</v>
+      </c>
+      <c r="I48" s="76">
+        <v>198.0</v>
+      </c>
+      <c r="J48" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="K48" s="74"/>
+    </row>
+    <row r="49" ht="15" customHeight="true">
+      <c r="A49" s="74" t="s">
+        <v>962</v>
+      </c>
+      <c r="B49" s="74" t="s">
+        <v>975</v>
+      </c>
+      <c r="C49" s="75">
+        <v>46065</v>
+      </c>
+      <c r="D49" s="74" t="s">
+        <v>429</v>
+      </c>
+      <c r="E49" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="F49" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G49" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H49" s="76">
+        <v>35.0</v>
+      </c>
+      <c r="I49" s="76">
+        <v>35.0</v>
+      </c>
+      <c r="J49" s="74" t="s">
+        <v>762</v>
+      </c>
+      <c r="K49" s="74"/>
+    </row>
+    <row r="50" ht="15" customHeight="true">
+      <c r="A50" s="74" t="s">
+        <v>962</v>
+      </c>
+      <c r="B50" s="74" t="s">
+        <v>975</v>
+      </c>
+      <c r="C50" s="75">
+        <v>46065</v>
+      </c>
+      <c r="D50" s="74" t="s">
+        <v>429</v>
+      </c>
+      <c r="E50" s="74" t="s">
+        <v>999</v>
+      </c>
+      <c r="F50" s="74" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G50" s="78">
+        <v>1.0</v>
+      </c>
+      <c r="H50" s="76">
+        <v>70.0</v>
+      </c>
+      <c r="I50" s="76">
+        <v>70.0</v>
+      </c>
+      <c r="J50" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="K50" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A46:C46"/>
+  </mergeCells>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
@@ -9810,134 +11623,289 @@
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="35"/>
-      <c r="B96" s="36"/>
-      <c r="C96" s="35"/>
-      <c r="D96" s="35"/>
-      <c r="E96" s="35"/>
-      <c r="F96" s="35"/>
-      <c r="G96" s="35"/>
-      <c r="H96" s="35"/>
+      <c r="A96" s="26" t="s">
+        <v>910</v>
+      </c>
+      <c r="B96" s="27">
+        <v>46074</v>
+      </c>
+      <c r="C96" s="28" t="s">
+        <v>915</v>
+      </c>
+      <c r="D96" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="E96" s="29" t="s">
+        <v>916</v>
+      </c>
+      <c r="F96" s="28" t="s">
+        <v>215</v>
+      </c>
+      <c r="G96" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H96" s="26">
+        <v>318</v>
+      </c>
       <c r="I96" s="35"/>
-      <c r="J96" s="35"/>
-      <c r="K96" s="35"/>
-      <c r="L96" s="11"/>
-      <c r="M96" s="11"/>
-      <c r="N96" s="11"/>
-      <c r="O96" s="37"/>
-      <c r="P96" s="38" t="n">
+      <c r="J96" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K96" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="L96" s="30">
+        <v>387.5</v>
+      </c>
+      <c r="M96" s="30">
+        <v>69.75</v>
+      </c>
+      <c r="N96" s="30">
+        <v>457.25</v>
+      </c>
+      <c r="O96" s="31">
+        <v>0</v>
+      </c>
+      <c r="P96" s="32">
         <f aca="false">N96-O96</f>
+      </c>
+      <c r="Q96" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R96" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="U96" s="29" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="26" t="s">
+        <v>911</v>
+      </c>
+      <c r="B97" s="27">
+        <v>46078</v>
+      </c>
+      <c r="C97" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="D97" s="28" t="s">
+        <v>920</v>
+      </c>
+      <c r="E97" s="29" t="s">
+        <v>921</v>
+      </c>
+      <c r="F97" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="G97" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H97" s="35"/>
+      <c r="I97" s="26" t="s">
+        <v>952</v>
+      </c>
+      <c r="J97" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K97" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="L97" s="30">
+        <v>13609.16</v>
+      </c>
+      <c r="M97" s="30">
+        <v>2449.65</v>
+      </c>
+      <c r="N97" s="30">
+        <v>16058.81</v>
+      </c>
+      <c r="O97" s="31">
+        <v>16058.81</v>
+      </c>
+      <c r="P97" s="32">
+        <f aca="false">N97-O97</f>
+      </c>
+      <c r="Q97" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="R97" s="28" t="s">
+        <v>854</v>
+      </c>
+      <c r="U97" s="29" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="26" t="s">
+        <v>912</v>
+      </c>
+      <c r="B98" s="27">
+        <v>46076</v>
+      </c>
+      <c r="C98" s="28" t="s">
+        <v>922</v>
+      </c>
+      <c r="D98" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="E98" s="29" t="s">
+        <v>923</v>
+      </c>
+      <c r="F98" s="28" t="s">
+        <v>924</v>
+      </c>
+      <c r="G98" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H98" s="26">
+        <v>323</v>
+      </c>
+      <c r="I98" s="35"/>
+      <c r="J98" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K98" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="L98" s="30">
+        <v>20986.2</v>
+      </c>
+      <c r="M98" s="30">
+        <v>3777.52</v>
+      </c>
+      <c r="N98" s="30">
+        <v>24763.72</v>
+      </c>
+      <c r="O98" s="31">
         <v>0</v>
       </c>
-      <c r="Q96" s="35"/>
-      <c r="R96" s="35"/>
-      <c r="S96" s="39"/>
-      <c r="T96" s="40"/>
-      <c r="U96" s="35"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="35"/>
-      <c r="B97" s="36"/>
-      <c r="C97" s="35"/>
-      <c r="D97" s="35"/>
-      <c r="E97" s="35"/>
-      <c r="F97" s="35"/>
-      <c r="G97" s="35"/>
-      <c r="H97" s="35"/>
-      <c r="I97" s="35"/>
-      <c r="J97" s="35"/>
-      <c r="K97" s="35"/>
-      <c r="L97" s="11"/>
-      <c r="M97" s="11"/>
-      <c r="N97" s="11"/>
-      <c r="O97" s="37"/>
-      <c r="P97" s="38" t="n">
-        <f aca="false">N97-O97</f>
+      <c r="P98" s="32">
+        <f aca="false">N98-O98</f>
+      </c>
+      <c r="Q98" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R98" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="U98" s="29" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="26" t="s">
+        <v>913</v>
+      </c>
+      <c r="B99" s="27">
+        <v>46079</v>
+      </c>
+      <c r="C99" s="28" t="s">
+        <v>925</v>
+      </c>
+      <c r="D99" s="28" t="s">
+        <v>926</v>
+      </c>
+      <c r="E99" s="29" t="s">
+        <v>927</v>
+      </c>
+      <c r="F99" s="28" t="s">
+        <v>928</v>
+      </c>
+      <c r="G99" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H99" s="26">
+        <v>324</v>
+      </c>
+      <c r="I99" s="35"/>
+      <c r="J99" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K99" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="L99" s="30">
+        <v>4300.0</v>
+      </c>
+      <c r="M99" s="30">
+        <v>774.0</v>
+      </c>
+      <c r="N99" s="30">
+        <v>5074.0</v>
+      </c>
+      <c r="O99" s="31">
         <v>0</v>
       </c>
-      <c r="Q97" s="35"/>
-      <c r="R97" s="35"/>
-      <c r="S97" s="39"/>
-      <c r="T97" s="40"/>
-      <c r="U97" s="35"/>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="35"/>
-      <c r="B98" s="36"/>
-      <c r="C98" s="35"/>
-      <c r="D98" s="35"/>
-      <c r="E98" s="35"/>
-      <c r="F98" s="35"/>
-      <c r="G98" s="35"/>
-      <c r="H98" s="35"/>
-      <c r="I98" s="35"/>
-      <c r="J98" s="35"/>
-      <c r="K98" s="35"/>
-      <c r="L98" s="11"/>
-      <c r="M98" s="11"/>
-      <c r="N98" s="11"/>
-      <c r="O98" s="37"/>
-      <c r="P98" s="38" t="n">
-        <f aca="false">N98-O98</f>
+      <c r="P99" s="32">
+        <f aca="false">N99-O99</f>
+      </c>
+      <c r="Q99" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R99" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="U99" s="29" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="26" t="s">
+        <v>914</v>
+      </c>
+      <c r="B100" s="27">
+        <v>46079</v>
+      </c>
+      <c r="C100" s="28" t="s">
+        <v>925</v>
+      </c>
+      <c r="D100" s="28" t="s">
+        <v>926</v>
+      </c>
+      <c r="E100" s="29" t="s">
+        <v>929</v>
+      </c>
+      <c r="F100" s="28" t="s">
+        <v>930</v>
+      </c>
+      <c r="G100" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H100" s="26">
+        <v>325</v>
+      </c>
+      <c r="I100" s="35"/>
+      <c r="J100" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K100" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="L100" s="30">
+        <v>6680.0</v>
+      </c>
+      <c r="M100" s="30">
+        <v>1202.4</v>
+      </c>
+      <c r="N100" s="30">
+        <v>7882.4</v>
+      </c>
+      <c r="O100" s="31">
         <v>0</v>
       </c>
-      <c r="Q98" s="35"/>
-      <c r="R98" s="35"/>
-      <c r="S98" s="39"/>
-      <c r="T98" s="40"/>
-      <c r="U98" s="35"/>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="35"/>
-      <c r="B99" s="36"/>
-      <c r="C99" s="35"/>
-      <c r="D99" s="35"/>
-      <c r="E99" s="35"/>
-      <c r="F99" s="35"/>
-      <c r="G99" s="35"/>
-      <c r="H99" s="35"/>
-      <c r="I99" s="35"/>
-      <c r="J99" s="35"/>
-      <c r="K99" s="35"/>
-      <c r="L99" s="11"/>
-      <c r="M99" s="11"/>
-      <c r="N99" s="11"/>
-      <c r="O99" s="37"/>
-      <c r="P99" s="38" t="n">
-        <f aca="false">N99-O99</f>
-        <v>0</v>
-      </c>
-      <c r="Q99" s="35"/>
-      <c r="R99" s="35"/>
-      <c r="S99" s="39"/>
-      <c r="T99" s="40"/>
-      <c r="U99" s="35"/>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="35"/>
-      <c r="B100" s="36"/>
-      <c r="C100" s="35"/>
-      <c r="D100" s="35"/>
-      <c r="E100" s="35"/>
-      <c r="F100" s="35"/>
-      <c r="G100" s="35"/>
-      <c r="H100" s="35"/>
-      <c r="I100" s="35"/>
-      <c r="J100" s="35"/>
-      <c r="K100" s="35"/>
-      <c r="L100" s="11"/>
-      <c r="M100" s="11"/>
-      <c r="N100" s="11"/>
-      <c r="O100" s="37"/>
-      <c r="P100" s="38" t="n">
+      <c r="P100" s="32">
         <f aca="false">N100-O100</f>
-        <v>0</v>
-      </c>
-      <c r="Q100" s="35"/>
-      <c r="R100" s="35"/>
-      <c r="S100" s="39"/>
-      <c r="T100" s="40"/>
-      <c r="U100" s="35"/>
+      </c>
+      <c r="Q100" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="R100" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="U100" s="29" t="s">
+        <v>931</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="35"/>
@@ -14542,24 +16510,158 @@
         <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B45,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>932</v>
+      </c>
+      <c r="B46" t="s">
+        <v>200</v>
+      </c>
+      <c r="C46" t="s">
+        <v>536</v>
+      </c>
+      <c r="D46" t="s">
+        <v>920</v>
+      </c>
+      <c r="F46" t="s">
+        <v>951</v>
+      </c>
+      <c r="G46">
+        <v>46078</v>
+      </c>
+      <c r="H46">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B46)</f>
+      </c>
+      <c r="I46">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B46,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J46">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B46,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B46,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K46">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B46)</f>
+      </c>
+      <c r="L46">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B46,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B46,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>933</v>
+      </c>
+      <c r="B47" t="s">
+        <v>922</v>
+      </c>
+      <c r="C47" t="s">
+        <v>936</v>
+      </c>
+      <c r="D47" t="s">
+        <v>163</v>
+      </c>
+      <c r="F47" t="s">
+        <v>506</v>
+      </c>
+      <c r="G47">
+        <v>46076</v>
+      </c>
+      <c r="H47">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B47)</f>
+      </c>
+      <c r="I47">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B47,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J47">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B47,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B47,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K47">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B47)</f>
+      </c>
+      <c r="L47">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B47,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B47,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>934</v>
+      </c>
+      <c r="B48" t="s">
+        <v>925</v>
+      </c>
+      <c r="D48" t="s">
+        <v>926</v>
+      </c>
+      <c r="F48" t="s">
+        <v>506</v>
+      </c>
+      <c r="G48">
+        <v>46079</v>
+      </c>
+      <c r="H48">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B48)</f>
+      </c>
+      <c r="I48">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B48,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J48">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B48,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B48,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K48">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B48)</f>
+      </c>
+      <c r="L48">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B48,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B48,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>935</v>
+      </c>
+      <c r="B49" t="s">
+        <v>915</v>
+      </c>
+      <c r="D49" t="s">
+        <v>69</v>
+      </c>
+      <c r="F49" t="s">
+        <v>506</v>
+      </c>
+      <c r="G49">
+        <v>46074</v>
+      </c>
+      <c r="H49">
+        <f>COUNTIF('Orders &amp; Payments'!$C$3:$C$200,$B49)</f>
+      </c>
+      <c r="I49">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Quotation")</f>
+      </c>
+      <c r="J49">
+        <f>SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$N$3:$N$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+      <c r="K49">
+        <f>SUMIFS('Orders &amp; Payments'!$O$3:$O$200,'Orders &amp; Payments'!$C$3:$C$200,$B49)</f>
+      </c>
+      <c r="L49">
+        <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
+      </c>
+    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H46" s="51" t="s">
+      <c r="H50" s="51" t="s">
         <v>446</v>
       </c>
-      <c r="I46" s="52" t="n">
-        <f aca="false">SUM(I3:I45)</f>
+      <c r="I50" s="52" t="n">
+        <f aca="false">SUM(I3:I49)</f>
         <v>286888.31</v>
       </c>
-      <c r="J46" s="52" t="n">
-        <f aca="false">SUM(J3:J45)</f>
+      <c r="J50" s="52" t="n">
+        <f aca="false">SUM(J3:J49)</f>
         <v>139259.89</v>
       </c>
-      <c r="K46" s="52" t="n">
-        <f aca="false">SUM(K3:K45)</f>
+      <c r="K50" s="52" t="n">
+        <f aca="false">SUM(K3:K49)</f>
         <v>12372.58</v>
       </c>
-      <c r="L46" s="52" t="n">
-        <f aca="false">SUM(L3:L45)</f>
+      <c r="L50" s="52" t="n">
+        <f aca="false">SUM(L3:L49)</f>
         <v>126887.31</v>
       </c>
     </row>
@@ -16262,45 +18364,145 @@
         <v>909</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="35"/>
-      <c r="B43" s="36"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="39"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="35"/>
-      <c r="H43" s="40"/>
-      <c r="I43" s="35"/>
-      <c r="J43" s="11"/>
-      <c r="K43" s="11" t="str">
-        <f aca="false">IF(J43="","",ROUND(J43*$R$2,2))</f>
-        <v/>
-      </c>
-      <c r="L43" s="35"/>
-      <c r="M43" s="39"/>
-      <c r="N43" s="40"/>
-      <c r="O43" s="35"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="35"/>
-      <c r="B44" s="36"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="40"/>
-      <c r="I44" s="35"/>
-      <c r="J44" s="11"/>
-      <c r="K44" s="11" t="str">
-        <f aca="false">IF(J44="","",ROUND(J44*$R$2,2))</f>
-        <v/>
-      </c>
-      <c r="L44" s="35"/>
-      <c r="M44" s="39"/>
-      <c r="N44" s="40"/>
-      <c r="O44" s="35"/>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>938</v>
+      </c>
+      <c r="B43">
+        <v>46074</v>
+      </c>
+      <c r="C43" t="s">
+        <v>915</v>
+      </c>
+      <c r="E43" t="s">
+        <v>69</v>
+      </c>
+      <c r="F43" t="s">
+        <v>916</v>
+      </c>
+      <c r="G43" t="s">
+        <v>609</v>
+      </c>
+      <c r="I43">
+        <v>318</v>
+      </c>
+      <c r="J43">
+        <v>457.25</v>
+      </c>
+      <c r="K43">
+        <f>IF(J43="","",ROUND(J43*$R$2,2))</f>
+      </c>
+      <c r="L43" t="s">
+        <v>49</v>
+      </c>
+      <c r="O43" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>939</v>
+      </c>
+      <c r="B44">
+        <v>46076</v>
+      </c>
+      <c r="C44" t="s">
+        <v>922</v>
+      </c>
+      <c r="E44" t="s">
+        <v>163</v>
+      </c>
+      <c r="F44" t="s">
+        <v>923</v>
+      </c>
+      <c r="G44" t="s">
+        <v>609</v>
+      </c>
+      <c r="I44">
+        <v>323</v>
+      </c>
+      <c r="J44">
+        <v>24763.72</v>
+      </c>
+      <c r="K44">
+        <f>IF(J44="","",ROUND(J44*$R$2,2))</f>
+      </c>
+      <c r="L44" t="s">
+        <v>49</v>
+      </c>
+      <c r="O44" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>940</v>
+      </c>
+      <c r="B45">
+        <v>46079</v>
+      </c>
+      <c r="C45" t="s">
+        <v>925</v>
+      </c>
+      <c r="E45" t="s">
+        <v>926</v>
+      </c>
+      <c r="F45" t="s">
+        <v>927</v>
+      </c>
+      <c r="G45" t="s">
+        <v>609</v>
+      </c>
+      <c r="I45">
+        <v>324</v>
+      </c>
+      <c r="J45">
+        <v>5074.0</v>
+      </c>
+      <c r="K45">
+        <f>IF(J45="","",ROUND(J45*$R$2,2))</f>
+      </c>
+      <c r="L45" t="s">
+        <v>49</v>
+      </c>
+      <c r="O45" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>941</v>
+      </c>
+      <c r="B46">
+        <v>46079</v>
+      </c>
+      <c r="C46" t="s">
+        <v>925</v>
+      </c>
+      <c r="E46" t="s">
+        <v>926</v>
+      </c>
+      <c r="F46" t="s">
+        <v>929</v>
+      </c>
+      <c r="G46" t="s">
+        <v>609</v>
+      </c>
+      <c r="I46">
+        <v>325</v>
+      </c>
+      <c r="J46">
+        <v>7882.4</v>
+      </c>
+      <c r="K46">
+        <f>IF(J46="","",ROUND(J46*$R$2,2))</f>
+      </c>
+      <c r="L46" t="s">
+        <v>49</v>
+      </c>
+      <c r="O46" t="s">
+        <v>931</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="35"/>

</xml_diff>

<commit_message>
Add batch 3 docs (MD-094–098) and Price Book tab
Orders & Payments:
- MD-094 MARSA: Quotation 318, Crema Galala Sills, €457.25 incl VAT
- MD-095 JAA CO LTD: Delivery-Invoice 1000302, Supply of Marble, €16,058.81 incl VAT
- MD-096 Gordon Vella: Quotation 323, Light Travertine Sills, €24,763.72 incl VAT
- MD-097 BJORN: Quotation 324, Bianco Marble & Nero Assaluto, €5,074.00 incl VAT
- MD-098 BJORN: Quotation 325, Quarzite & Crema Marfil, €7,882.40 incl VAT

Client Directory: C-044 JAA CO LTD, C-045 Gordon Vella, C-046 BJORN, C-047 MARSA
Measurement Pipeline: L-041 to L-044 for all 4 open quotes

New Price Book tab (tab 10): 13 client sections, 35 line items extracted
from all PDFs — material, unit, qty, unit price per client for quick reference

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6MGCGosiZzZvgoKjqDuZ7
</commit_message>
<xml_diff>
--- a/MD_Marble_Factory_Tracker_Updated.xlsx
+++ b/MD_Marble_Factory_Tracker_Updated.xlsx
@@ -16644,7 +16644,7 @@
         <f>SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Invoice")+SUMIFS('Orders &amp; Payments'!$P$3:$P$200,'Orders &amp; Payments'!$C$3:$C$200,$B49,'Orders &amp; Payments'!$G$3:$G$200,"Delivery-Invoice")</f>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H50" s="51" t="s">
         <v>446</v>
       </c>
@@ -18503,46 +18503,6 @@
       <c r="O46" t="s">
         <v>931</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="35"/>
-      <c r="B45" s="36"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="35"/>
-      <c r="J45" s="11"/>
-      <c r="K45" s="11" t="str">
-        <f aca="false">IF(J45="","",ROUND(J45*$R$2,2))</f>
-        <v/>
-      </c>
-      <c r="L45" s="35"/>
-      <c r="M45" s="39"/>
-      <c r="N45" s="40"/>
-      <c r="O45" s="35"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35"/>
-      <c r="B46" s="36"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="40"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="11"/>
-      <c r="K46" s="11" t="str">
-        <f aca="false">IF(J46="","",ROUND(J46*$R$2,2))</f>
-        <v/>
-      </c>
-      <c r="L46" s="35"/>
-      <c r="M46" s="39"/>
-      <c r="N46" s="40"/>
-      <c r="O46" s="35"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="35"/>

</xml_diff>

<commit_message>
Batch 7: ST Projects Galal Marble Gzira Inv 1000309 (MD-108)
</commit_message>
<xml_diff>
--- a/MD_Marble_Factory_Tracker_Updated.xlsx
+++ b/MD_Marble_Factory_Tracker_Updated.xlsx
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="1111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="1135">
   <si>
     <t>MD MARBLE  —  FACTORY CONTROL DASHBOARD</t>
   </si>
@@ -3512,6 +3512,15 @@
   </si>
   <si>
     <t>Installation of Staircase 2</t>
+  </si>
+  <si>
+    <t>MD-108</t>
+  </si>
+  <si>
+    <t>Supply of Galal Marble Gzira (widths: up to 30cm, 32cm, 43cm)</t>
+  </si>
+  <si>
+    <t>Supply only — Balance due €5,370.08</t>
   </si>
 </sst>
 </file>
@@ -13970,6 +13979,57 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" t="s" s="26">
+        <v>1132</v>
+      </c>
+      <c r="B108" s="27">
+        <v>46090</v>
+      </c>
+      <c r="C108" t="s" s="28">
+        <v>1055</v>
+      </c>
+      <c r="D108" t="s" s="28">
+        <v>1078</v>
+      </c>
+      <c r="E108" t="s" s="29">
+        <v>1133</v>
+      </c>
+      <c r="F108" t="s" s="28">
+        <v>1058</v>
+      </c>
+      <c r="G108" t="s" s="26">
+        <v>18</v>
+      </c>
+      <c r="I108" s="35">
+        <v>1000309</v>
+      </c>
+      <c r="J108" t="s" s="28">
+        <v>15</v>
+      </c>
+      <c r="L108" s="30">
+        <v>4550.92</v>
+      </c>
+      <c r="M108" s="30">
+        <v>819.16</v>
+      </c>
+      <c r="N108" s="30">
+        <v>5370.08</v>
+      </c>
+      <c r="O108" s="31">
+        <v>0</v>
+      </c>
+      <c r="P108" s="32">
+        <f>N108-O108</f>
+        <v>5370.08</v>
+      </c>
+      <c r="R108" t="s" s="28">
+        <v>854</v>
+      </c>
+      <c r="U108" t="s" s="29">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="35"/>
       <c r="B108" s="36"/>
       <c r="C108" s="35"/>

</xml_diff>